<commit_message>
two quesition day 12
</commit_message>
<xml_diff>
--- a/NeetCode_150_FAANG_Tracker.xlsx
+++ b/NeetCode_150_FAANG_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/faizan/faizan/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCCFF84E-5B4F-2E41-B34C-89CCC59A0425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24ACBC7E-89B1-3444-8707-3D0BA04D1BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="141">
   <si>
     <t>Order</t>
   </si>
@@ -426,6 +426,24 @@
   </si>
   <si>
     <t>day10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">solve by help using striver same two pointer using leftMax and rmax </t>
+  </si>
+  <si>
+    <t>day 11</t>
+  </si>
+  <si>
+    <t>day11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">done but not solve by own buy and sell variable are used to do it and using while maximumly when we have two pointer and sw </t>
+  </si>
+  <si>
+    <t>start= Math.max(start,map.get(s[end])+1),maxLen = Math.max(maxLen, end - start + 1);</t>
+  </si>
+  <si>
+    <t>day12</t>
   </si>
 </sst>
 </file>
@@ -775,7 +793,8 @@
   <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="23.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="3" max="3" width="38.1640625" customWidth="1"/>
     <col min="4" max="4" width="17.1640625" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="7" max="7" width="18.1640625" customWidth="1"/>
@@ -1114,7 +1133,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>46047</v>
       </c>
@@ -1131,10 +1150,19 @@
         <v>20</v>
       </c>
       <c r="F14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+      <c r="G14" t="s">
+        <v>108</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>46048</v>
+      </c>
       <c r="B15">
         <v>14</v>
       </c>
@@ -1147,8 +1175,20 @@
       <c r="E15" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F15" t="s">
+        <v>136</v>
+      </c>
+      <c r="G15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>46048</v>
+      </c>
       <c r="B16">
         <v>15</v>
       </c>
@@ -1161,8 +1201,20 @@
       <c r="E16" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>136</v>
+      </c>
+      <c r="G16" t="s">
+        <v>108</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>46049</v>
+      </c>
       <c r="B17">
         <v>16</v>
       </c>
@@ -1175,8 +1227,11 @@
       <c r="E17" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B18">
         <v>17</v>
       </c>
@@ -1190,7 +1245,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B19">
         <v>18</v>
       </c>
@@ -1204,7 +1259,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B20">
         <v>19</v>
       </c>
@@ -1218,7 +1273,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B21">
         <v>20</v>
       </c>
@@ -1232,7 +1287,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B22">
         <v>21</v>
       </c>
@@ -1246,7 +1301,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B23">
         <v>22</v>
       </c>
@@ -1260,7 +1315,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B24">
         <v>23</v>
       </c>
@@ -1274,7 +1329,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B25">
         <v>24</v>
       </c>
@@ -1288,7 +1343,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B26">
         <v>25</v>
       </c>
@@ -1302,7 +1357,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B27">
         <v>26</v>
       </c>
@@ -1316,7 +1371,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B28">
         <v>27</v>
       </c>
@@ -1330,7 +1385,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B29">
         <v>28</v>
       </c>
@@ -1344,7 +1399,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B30">
         <v>29</v>
       </c>
@@ -1358,7 +1413,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B31">
         <v>30</v>
       </c>
@@ -1372,7 +1427,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B32">
         <v>31</v>
       </c>

</xml_diff>